<commit_message>
chore: permanently remove teacher-sqa folder
</commit_message>
<xml_diff>
--- a/Testcase_templateLab3_673380602-6.xlsx
+++ b/Testcase_templateLab3_673380602-6.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kkumail-my.sharepoint.com/personal/sasiwitra_w_kkumail_com/Documents/kku study/LAB/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/inzi/Lab3SQA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="8_{49B13566-DA13-3047-9FA2-C215C8121EC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87E7F5A7-672F-424E-B304-5F7C7AC428B4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8B9BAB0C-57B6-6240-A93E-2D965683EA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="16060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="16060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenario Summary" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="90">
   <si>
     <t>Scenario ID</t>
   </si>
@@ -257,9 +257,6 @@
     <t>software</t>
   </si>
   <si>
-    <t>เมธอด return ผลลัพธ์เป็น "zvmadhyl"</t>
-  </si>
-  <si>
     <t>TC03</t>
   </si>
   <si>
@@ -282,6 +279,36 @@
   </si>
   <si>
     <t>pass</t>
+  </si>
+  <si>
+    <t>DF001</t>
+  </si>
+  <si>
+    <t>Shift method returns "invalid" when input contains special characters or spaces</t>
+  </si>
+  <si>
+    <t>673380602-6</t>
+  </si>
+  <si>
+    <t>เมื่อเรียกใช้เมธอด shift() โดยส่งข้อความที่มีช่องว่างหรือสัญลักษณ์พิเศษ เช่น "SQA #1" และคีย์เป็น 3 ตัวโปรแกรมควรจะเลื่อนตัวอักษรและคงอักขระพิเศษไว้ (Expected: "ZXH #1") แต่ระบบกลับส่งค่าคืนมาเป็น "invalid" (Actual: "invalid")</t>
+  </si>
+  <si>
+    <t>Sqa2026</t>
+  </si>
+  <si>
+    <t>SQA #1</t>
+  </si>
+  <si>
+    <t>เมธอด return ผลลัพธ์เป็น "invalid"</t>
+  </si>
+  <si>
+    <t>เมธอด return ผลลัพธ์เป็น "ZXH #1"</t>
+  </si>
+  <si>
+    <t>"ZVMADHYL"</t>
+  </si>
+  <si>
+    <t>"invalid"</t>
   </si>
 </sst>
 </file>
@@ -516,7 +543,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -697,6 +724,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -1033,9 +1064,15 @@
       <c r="C3" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
+      <c r="D3" s="22">
+        <v>4</v>
+      </c>
+      <c r="E3" s="22">
+        <v>3</v>
+      </c>
+      <c r="F3" s="22">
+        <v>1</v>
+      </c>
       <c r="G3" s="22"/>
       <c r="H3" s="22"/>
       <c r="I3" s="25" t="s">
@@ -1092,9 +1129,15 @@
       </c>
       <c r="B8" s="51"/>
       <c r="C8" s="52"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="27"/>
+      <c r="D8" s="13">
+        <v>4</v>
+      </c>
+      <c r="E8" s="26">
+        <v>3</v>
+      </c>
+      <c r="F8" s="27">
+        <v>1</v>
+      </c>
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
       <c r="I8" s="28" t="s">
@@ -1140,7 +1183,7 @@
         <v>23</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>24</v>
@@ -1149,7 +1192,7 @@
         <v>25</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>26</v>
@@ -1164,23 +1207,33 @@
         <v>29</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="24" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="175" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
+      <c r="B3" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" s="66" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" s="2">
+        <v>46210</v>
+      </c>
       <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
+      <c r="F3" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
+      <c r="K3" s="66" t="s">
+        <v>83</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1514,10 +1567,10 @@
       <c r="C5" s="39"/>
       <c r="D5" s="39"/>
       <c r="E5" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="38" t="s">
         <v>75</v>
-      </c>
-      <c r="F5" s="38" t="s">
-        <v>76</v>
       </c>
       <c r="G5" s="42"/>
     </row>
@@ -1582,9 +1635,11 @@
       <c r="E10" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="F10" s="13"/>
+      <c r="F10" s="13" t="s">
+        <v>88</v>
+      </c>
       <c r="G10" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.4">
@@ -1599,37 +1654,55 @@
         <v>3</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="F11" s="13"/>
+        <v>86</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>89</v>
+      </c>
       <c r="G11" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="36"/>
       <c r="B12" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
+        <v>72</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" s="13">
+        <v>3</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="F12" t="s">
+        <v>89</v>
+      </c>
       <c r="G12" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="37"/>
       <c r="B13" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13"/>
-      <c r="F13" s="13"/>
+        <v>73</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="13">
+        <v>3</v>
+      </c>
+      <c r="E13" s="67" t="s">
+        <v>87</v>
+      </c>
+      <c r="F13" t="s">
+        <v>89</v>
+      </c>
       <c r="G13" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update test cases and template spreadsheet
</commit_message>
<xml_diff>
--- a/Testcase_templateLab3_673380602-6.xlsx
+++ b/Testcase_templateLab3_673380602-6.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/inzi/Lab3SQA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kkumail-my.sharepoint.com/personal/sasiwitra_w_kkumail_com/Documents/kku study/LAB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8B9BAB0C-57B6-6240-A93E-2D965683EA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{3D836475-9685-314E-A529-53DA6AA968FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="16060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="89">
   <si>
     <t>Scenario ID</t>
   </si>
@@ -269,6 +269,12 @@
     <t>ศศิวิตรา วงษ์รุ่งอรุณเลิศ 673380602-6</t>
   </si>
   <si>
+    <t>Sqa2026</t>
+  </si>
+  <si>
+    <t>SQA #1</t>
+  </si>
+  <si>
     <t>Reporter ใครรายงาน</t>
   </si>
   <si>
@@ -278,7 +284,30 @@
     <t>Defect Title ชื่อ</t>
   </si>
   <si>
-    <t>pass</t>
+    <t>673380602-6</t>
+  </si>
+  <si>
+    <t>"invalid"</t>
+  </si>
+  <si>
+    <t>"ZVMADHYL"</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">เมธอด return ผลลัพธ์เป็น </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>"ZXH #1"</t>
+    </r>
+  </si>
+  <si>
+    <t>เมธอด return ผลลัพธ์เป็น "invalid"</t>
   </si>
   <si>
     <t>DF001</t>
@@ -287,35 +316,14 @@
     <t>Shift method returns "invalid" when input contains special characters or spaces</t>
   </si>
   <si>
-    <t>673380602-6</t>
-  </si>
-  <si>
     <t>เมื่อเรียกใช้เมธอด shift() โดยส่งข้อความที่มีช่องว่างหรือสัญลักษณ์พิเศษ เช่น "SQA #1" และคีย์เป็น 3 ตัวโปรแกรมควรจะเลื่อนตัวอักษรและคงอักขระพิเศษไว้ (Expected: "ZXH #1") แต่ระบบกลับส่งค่าคืนมาเป็น "invalid" (Actual: "invalid")</t>
-  </si>
-  <si>
-    <t>Sqa2026</t>
-  </si>
-  <si>
-    <t>SQA #1</t>
-  </si>
-  <si>
-    <t>เมธอด return ผลลัพธ์เป็น "invalid"</t>
-  </si>
-  <si>
-    <t>เมธอด return ผลลัพธ์เป็น "ZXH #1"</t>
-  </si>
-  <si>
-    <t>"ZVMADHYL"</t>
-  </si>
-  <si>
-    <t>"invalid"</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -394,6 +402,12 @@
       <name val="TH SarabunPSK"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -543,7 +557,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -620,25 +634,79 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -646,12 +714,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -665,69 +727,17 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -1061,7 +1071,7 @@
       <c r="B3" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="32" t="s">
         <v>56</v>
       </c>
       <c r="D3" s="22">
@@ -1124,11 +1134,11 @@
       <c r="I7" s="13"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.4">
-      <c r="A8" s="50" t="s">
+      <c r="A8" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="51"/>
-      <c r="C8" s="52"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="36"/>
       <c r="D8" s="13">
         <v>4</v>
       </c>
@@ -1138,8 +1148,12 @@
       <c r="F8" s="27">
         <v>1</v>
       </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
+      <c r="G8" s="13">
+        <v>0</v>
+      </c>
+      <c r="H8" s="13">
+        <v>0</v>
+      </c>
       <c r="I8" s="28" t="s">
         <v>18</v>
       </c>
@@ -1183,7 +1197,7 @@
         <v>23</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>24</v>
@@ -1192,7 +1206,7 @@
         <v>25</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>26</v>
@@ -1207,32 +1221,32 @@
         <v>29</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="175" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3" s="66" t="s">
-        <v>81</v>
+      <c r="B3" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="33" t="s">
+        <v>87</v>
       </c>
       <c r="D3" s="2">
         <v>46210</v>
       </c>
-      <c r="E3" s="1"/>
+      <c r="E3" s="2"/>
       <c r="F3" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="66" t="s">
-        <v>83</v>
+      <c r="K3" s="33" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1266,10 +1280,10 @@
       <c r="C1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="40" t="s">
+      <c r="D1" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="E1" s="41"/>
+      <c r="E1" s="39"/>
     </row>
     <row r="2" spans="1:8" ht="56" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
@@ -1281,10 +1295,10 @@
       <c r="C2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="40" t="s">
+      <c r="D2" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="41"/>
+      <c r="E2" s="39"/>
     </row>
     <row r="3" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
@@ -1294,10 +1308,10 @@
       <c r="C3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="41"/>
+      <c r="E3" s="39"/>
     </row>
     <row r="4" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
@@ -1309,39 +1323,39 @@
       <c r="C4" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="53"/>
-      <c r="E4" s="53"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
     </row>
     <row r="5" spans="1:8" ht="28" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="62" t="s">
+      <c r="B5" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="62"/>
-      <c r="D5" s="62"/>
-      <c r="E5" s="62"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
     </row>
     <row r="6" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="48" t="s">
         <v>68</v>
       </c>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
     </row>
     <row r="7" spans="1:8" ht="27" x14ac:dyDescent="0.45">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="61"/>
-      <c r="C7" s="61"/>
-      <c r="D7" s="61"/>
-      <c r="E7" s="61"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
     </row>
     <row r="8" spans="1:8" ht="27" x14ac:dyDescent="0.45">
       <c r="A8" s="7" t="s">
@@ -1370,10 +1384,10 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="51" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="63">
+      <c r="A9" s="49">
         <v>1</v>
       </c>
-      <c r="B9" s="55" t="s">
+      <c r="B9" s="41" t="s">
         <v>58</v>
       </c>
       <c r="C9" s="30" t="s">
@@ -1382,7 +1396,7 @@
       <c r="D9" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="58" t="s">
+      <c r="E9" s="44" t="s">
         <v>61</v>
       </c>
       <c r="F9" s="8"/>
@@ -1390,27 +1404,27 @@
       <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:8" ht="51" x14ac:dyDescent="0.45">
-      <c r="A10" s="64"/>
-      <c r="B10" s="56"/>
+      <c r="A10" s="50"/>
+      <c r="B10" s="42"/>
       <c r="C10" s="8" t="s">
         <v>57</v>
       </c>
       <c r="D10" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="E10" s="59"/>
+      <c r="E10" s="45"/>
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" ht="27" x14ac:dyDescent="0.45">
-      <c r="A11" s="65"/>
-      <c r="B11" s="57"/>
+      <c r="A11" s="51"/>
+      <c r="B11" s="43"/>
       <c r="C11" s="8"/>
       <c r="D11" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="E11" s="60"/>
+      <c r="E11" s="46"/>
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
@@ -1479,12 +1493,12 @@
       <c r="A18" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="54" t="s">
+      <c r="B18" s="40" t="s">
         <v>62</v>
       </c>
-      <c r="C18" s="54"/>
-      <c r="D18" s="54"/>
-      <c r="E18" s="54"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
     </row>
     <row r="19" spans="1:8" ht="27" x14ac:dyDescent="0.45">
       <c r="A19" s="10"/>
@@ -1530,179 +1544,179 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" s="17" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
     </row>
     <row r="4" spans="1:7" ht="27" x14ac:dyDescent="0.4">
       <c r="A4" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="56" t="s">
         <v>66</v>
       </c>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
       <c r="E4" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="40" t="s">
+      <c r="F4" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="G4" s="41"/>
+      <c r="G4" s="39"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="56" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
       <c r="E5" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="F5" s="38" t="s">
+      <c r="F5" s="56" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="42"/>
+      <c r="G5" s="58"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="43"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-      <c r="G6" s="45"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
+      <c r="G6" s="61"/>
     </row>
     <row r="8" spans="1:7" s="21" customFormat="1" ht="25" x14ac:dyDescent="0.2">
-      <c r="A8" s="48" t="s">
+      <c r="A8" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="48" t="s">
+      <c r="B8" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="46" t="s">
+      <c r="C8" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="47"/>
-      <c r="E8" s="48" t="s">
+      <c r="D8" s="63"/>
+      <c r="E8" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="48" t="s">
+      <c r="F8" s="64" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="20" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="49"/>
-      <c r="B9" s="49"/>
+    <row r="9" spans="1:7" s="21" customFormat="1" ht="25" x14ac:dyDescent="0.2">
+      <c r="A9" s="65"/>
+      <c r="B9" s="65"/>
       <c r="C9" s="31" t="s">
         <v>63</v>
       </c>
       <c r="D9" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="32"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A10" s="35" t="s">
+      <c r="E9" s="65"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="31"/>
+    </row>
+    <row r="10" spans="1:7" ht="25" x14ac:dyDescent="0.4">
+      <c r="A10" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="29">
         <v>3</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="F10" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="G10" s="13" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A11" s="36"/>
-      <c r="B11" s="13" t="s">
+      <c r="F10" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="G10" s="29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="25" x14ac:dyDescent="0.4">
+      <c r="A11" s="54"/>
+      <c r="B11" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="29">
         <v>3</v>
       </c>
-      <c r="E11" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A12" s="36"/>
-      <c r="B12" s="13" t="s">
+      <c r="E11" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="F11" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11" s="29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="25" x14ac:dyDescent="0.4">
+      <c r="A12" s="54"/>
+      <c r="B12" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12" s="29">
+        <v>3</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="F12" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="G12" s="29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="25" x14ac:dyDescent="0.4">
+      <c r="A13" s="55"/>
+      <c r="B13" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="C13" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13" s="29">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
         <v>84</v>
       </c>
-      <c r="D12" s="13">
-        <v>3</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F12" t="s">
-        <v>89</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A13" s="37"/>
-      <c r="B13" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="D13" s="13">
-        <v>3</v>
-      </c>
-      <c r="E13" s="67" t="s">
-        <v>87</v>
-      </c>
-      <c r="F13" t="s">
-        <v>89</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>79</v>
+      <c r="F13" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="G13" s="29" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>